<commit_message>
Cambio en archivo de resumen
</commit_message>
<xml_diff>
--- a/resumen_trabajos.xlsx
+++ b/resumen_trabajos.xlsx
@@ -1,21 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29401"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_FA6C15EC1F8105EF536CA9CD4AC80951B8751AF9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dacm/Proyectos_we/odoo_con_trabajos/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0AEEBC5-1C46-DD4D-B65A-914A85E774E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-228" yWindow="12852" windowWidth="23256" windowHeight="13896" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="provisoria" sheetId="1" r:id="rId1"/>
-    <sheet name="Capa_1" sheetId="2" r:id="rId2"/>
-    <sheet name="Capa_2" sheetId="3" r:id="rId3"/>
+    <sheet name="merge" sheetId="4" r:id="rId2"/>
+    <sheet name="Capa_1" sheetId="2" r:id="rId3"/>
+    <sheet name="Capa_2" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Capa_1!$A$1:$H$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Capa_2!$A$1:$L$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">provisoria!$A$1:$M$184</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Capa_1!$A$1:$H$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Capa_2!$A$1:$L$84</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -2348,7 +2354,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2727,23 +2733,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q184"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="67.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="67.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="37.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="94.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="96.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="255.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="94.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="96.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="255.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2788,7 +2794,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>144</v>
       </c>
@@ -2829,7 +2835,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>143</v>
       </c>
@@ -2858,7 +2864,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>139</v>
       </c>
@@ -2899,7 +2905,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>138</v>
       </c>
@@ -2928,7 +2934,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>136</v>
       </c>
@@ -2969,7 +2975,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>133</v>
       </c>
@@ -3007,7 +3013,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>132</v>
       </c>
@@ -3036,7 +3042,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>130</v>
       </c>
@@ -3065,7 +3071,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>130</v>
       </c>
@@ -3094,7 +3100,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>129</v>
       </c>
@@ -3123,7 +3129,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>129</v>
       </c>
@@ -3152,7 +3158,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>129</v>
       </c>
@@ -3181,7 +3187,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>129</v>
       </c>
@@ -3210,7 +3216,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>129</v>
       </c>
@@ -3239,7 +3245,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>129</v>
       </c>
@@ -3268,7 +3274,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>126</v>
       </c>
@@ -3297,7 +3303,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>126</v>
       </c>
@@ -3326,7 +3332,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>126</v>
       </c>
@@ -3355,7 +3361,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>125</v>
       </c>
@@ -3396,7 +3402,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>125</v>
       </c>
@@ -3437,7 +3443,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>124</v>
       </c>
@@ -3478,7 +3484,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>124</v>
       </c>
@@ -3519,7 +3525,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>123</v>
       </c>
@@ -3548,7 +3554,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>123</v>
       </c>
@@ -3577,7 +3583,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>123</v>
       </c>
@@ -3606,7 +3612,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>122</v>
       </c>
@@ -3644,7 +3650,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>122</v>
       </c>
@@ -3685,7 +3691,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>122</v>
       </c>
@@ -3723,7 +3729,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>122</v>
       </c>
@@ -3761,7 +3767,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>122</v>
       </c>
@@ -3799,7 +3805,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>121</v>
       </c>
@@ -3840,7 +3846,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>121</v>
       </c>
@@ -3881,7 +3887,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:13">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>120</v>
       </c>
@@ -3919,7 +3925,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>119</v>
       </c>
@@ -3957,7 +3963,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>119</v>
       </c>
@@ -3995,7 +4001,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>119</v>
       </c>
@@ -4033,7 +4039,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>119</v>
       </c>
@@ -4071,7 +4077,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>119</v>
       </c>
@@ -4112,7 +4118,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>118</v>
       </c>
@@ -4141,7 +4147,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:13">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>118</v>
       </c>
@@ -4170,7 +4176,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:13">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>118</v>
       </c>
@@ -4211,7 +4217,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:13">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>117</v>
       </c>
@@ -4252,7 +4258,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>117</v>
       </c>
@@ -4293,7 +4299,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:13">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>117</v>
       </c>
@@ -4322,7 +4328,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46" spans="1:13">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>116</v>
       </c>
@@ -4360,7 +4366,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:13">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>116</v>
       </c>
@@ -4398,7 +4404,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>115</v>
       </c>
@@ -4427,7 +4433,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:13">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>115</v>
       </c>
@@ -4456,7 +4462,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:13">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>115</v>
       </c>
@@ -4485,7 +4491,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51" spans="1:13">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>114</v>
       </c>
@@ -4514,7 +4520,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:13">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>114</v>
       </c>
@@ -4543,7 +4549,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:13">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>112</v>
       </c>
@@ -4572,7 +4578,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54" spans="1:13">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>112</v>
       </c>
@@ -4601,7 +4607,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:13">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>111</v>
       </c>
@@ -4630,7 +4636,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:13">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>111</v>
       </c>
@@ -4659,7 +4665,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:13">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>111</v>
       </c>
@@ -4688,7 +4694,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:13">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>110</v>
       </c>
@@ -4717,7 +4723,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="1:13">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>110</v>
       </c>
@@ -4746,7 +4752,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:13">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>110</v>
       </c>
@@ -4775,7 +4781,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:13">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>108</v>
       </c>
@@ -4813,7 +4819,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="62" spans="1:13">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>108</v>
       </c>
@@ -4851,7 +4857,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:13">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>106</v>
       </c>
@@ -4892,7 +4898,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="64" spans="1:13">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>105</v>
       </c>
@@ -4921,7 +4927,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="65" spans="1:13">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>105</v>
       </c>
@@ -4950,7 +4956,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:13">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>105</v>
       </c>
@@ -4988,7 +4994,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="67" spans="1:13">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>104</v>
       </c>
@@ -5026,7 +5032,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="1:13">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>103</v>
       </c>
@@ -5055,7 +5061,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="1:13">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>102</v>
       </c>
@@ -5084,7 +5090,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:13">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>101</v>
       </c>
@@ -5113,7 +5119,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="1:13">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>101</v>
       </c>
@@ -5142,7 +5148,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:13">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>101</v>
       </c>
@@ -5171,7 +5177,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="73" spans="1:13">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>101</v>
       </c>
@@ -5200,7 +5206,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="74" spans="1:13">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>101</v>
       </c>
@@ -5229,7 +5235,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:13">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>101</v>
       </c>
@@ -5270,7 +5276,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:13">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>100</v>
       </c>
@@ -5299,7 +5305,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="77" spans="1:13">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>100</v>
       </c>
@@ -5328,7 +5334,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="1:13">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>100</v>
       </c>
@@ -5357,7 +5363,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="1:13">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>100</v>
       </c>
@@ -5386,7 +5392,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:13">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>100</v>
       </c>
@@ -5415,7 +5421,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="81" spans="1:13">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>99</v>
       </c>
@@ -5456,7 +5462,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="1:13">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>98</v>
       </c>
@@ -5485,7 +5491,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:13">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>97</v>
       </c>
@@ -5514,7 +5520,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:13">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>97</v>
       </c>
@@ -5543,7 +5549,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:13">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>97</v>
       </c>
@@ -5584,7 +5590,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:13">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>96</v>
       </c>
@@ -5613,7 +5619,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="1:13">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>96</v>
       </c>
@@ -5651,7 +5657,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:13">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>96</v>
       </c>
@@ -5689,7 +5695,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="1:13">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>95</v>
       </c>
@@ -5718,7 +5724,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="90" spans="1:13">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>95</v>
       </c>
@@ -5756,7 +5762,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="91" spans="1:13">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>95</v>
       </c>
@@ -5794,7 +5800,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="92" spans="1:13">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>94</v>
       </c>
@@ -5823,7 +5829,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="93" spans="1:13">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>94</v>
       </c>
@@ -5852,7 +5858,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="94" spans="1:13">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>94</v>
       </c>
@@ -5881,7 +5887,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="95" spans="1:13">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>94</v>
       </c>
@@ -5910,7 +5916,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="96" spans="1:13">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>93</v>
       </c>
@@ -5939,7 +5945,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="97" spans="1:13">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>93</v>
       </c>
@@ -5968,7 +5974,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="98" spans="1:13">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>93</v>
       </c>
@@ -5997,7 +6003,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="99" spans="1:13">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>93</v>
       </c>
@@ -6026,7 +6032,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="100" spans="1:13">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>93</v>
       </c>
@@ -6067,7 +6073,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="101" spans="1:13">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>93</v>
       </c>
@@ -6108,7 +6114,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="102" spans="1:13">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>92</v>
       </c>
@@ -6137,7 +6143,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="103" spans="1:13">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>91</v>
       </c>
@@ -6166,7 +6172,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="104" spans="1:13">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>91</v>
       </c>
@@ -6207,7 +6213,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="105" spans="1:13">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>91</v>
       </c>
@@ -6248,7 +6254,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="1:13">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>91</v>
       </c>
@@ -6289,7 +6295,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:13">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>91</v>
       </c>
@@ -6330,7 +6336,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:13">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>90</v>
       </c>
@@ -6371,7 +6377,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="109" spans="1:13">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>89</v>
       </c>
@@ -6412,7 +6418,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="110" spans="1:13">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>89</v>
       </c>
@@ -6453,7 +6459,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="111" spans="1:13">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>88</v>
       </c>
@@ -6491,7 +6497,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="112" spans="1:13">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>88</v>
       </c>
@@ -6526,7 +6532,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="113" spans="1:13">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>87</v>
       </c>
@@ -6555,7 +6561,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="114" spans="1:13">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>86</v>
       </c>
@@ -6596,7 +6602,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="115" spans="1:13">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>86</v>
       </c>
@@ -6637,7 +6643,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="116" spans="1:13">
+    <row r="116" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>86</v>
       </c>
@@ -6678,7 +6684,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="117" spans="1:13">
+    <row r="117" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>86</v>
       </c>
@@ -6719,7 +6725,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="118" spans="1:13">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>86</v>
       </c>
@@ -6760,7 +6766,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="119" spans="1:13">
+    <row r="119" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>86</v>
       </c>
@@ -6801,7 +6807,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="120" spans="1:13">
+    <row r="120" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>84</v>
       </c>
@@ -6842,7 +6848,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="121" spans="1:13">
+    <row r="121" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>84</v>
       </c>
@@ -6883,7 +6889,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="122" spans="1:13">
+    <row r="122" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>83</v>
       </c>
@@ -6912,7 +6918,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="123" spans="1:13">
+    <row r="123" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>83</v>
       </c>
@@ -6953,7 +6959,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="124" spans="1:13">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>83</v>
       </c>
@@ -6994,7 +7000,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="125" spans="1:13">
+    <row r="125" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>83</v>
       </c>
@@ -7035,7 +7041,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="126" spans="1:13">
+    <row r="126" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>83</v>
       </c>
@@ -7073,7 +7079,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="127" spans="1:13">
+    <row r="127" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>82</v>
       </c>
@@ -7114,7 +7120,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="128" spans="1:13">
+    <row r="128" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>81</v>
       </c>
@@ -7143,7 +7149,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="129" spans="1:13">
+    <row r="129" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>81</v>
       </c>
@@ -7172,7 +7178,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="130" spans="1:13">
+    <row r="130" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>81</v>
       </c>
@@ -7213,7 +7219,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="131" spans="1:13">
+    <row r="131" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>81</v>
       </c>
@@ -7254,7 +7260,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="132" spans="1:13">
+    <row r="132" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>81</v>
       </c>
@@ -7292,7 +7298,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="133" spans="1:13">
+    <row r="133" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>81</v>
       </c>
@@ -7333,7 +7339,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="134" spans="1:13">
+    <row r="134" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>81</v>
       </c>
@@ -7371,7 +7377,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="135" spans="1:13">
+    <row r="135" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>81</v>
       </c>
@@ -7409,7 +7415,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="136" spans="1:13">
+    <row r="136" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>78</v>
       </c>
@@ -7438,7 +7444,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="137" spans="1:13">
+    <row r="137" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>76</v>
       </c>
@@ -7479,7 +7485,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="138" spans="1:13">
+    <row r="138" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>75</v>
       </c>
@@ -7508,7 +7514,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="139" spans="1:13">
+    <row r="139" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>74</v>
       </c>
@@ -7537,7 +7543,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="140" spans="1:13">
+    <row r="140" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>73</v>
       </c>
@@ -7578,7 +7584,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="141" spans="1:13">
+    <row r="141" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>73</v>
       </c>
@@ -7619,7 +7625,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="142" spans="1:13">
+    <row r="142" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>73</v>
       </c>
@@ -7660,7 +7666,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="143" spans="1:13">
+    <row r="143" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>72</v>
       </c>
@@ -7689,7 +7695,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="144" spans="1:13">
+    <row r="144" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>72</v>
       </c>
@@ -7718,7 +7724,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="145" spans="1:13">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>70</v>
       </c>
@@ -7756,7 +7762,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="146" spans="1:13">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>70</v>
       </c>
@@ -7794,7 +7800,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="147" spans="1:13">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>70</v>
       </c>
@@ -7832,7 +7838,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="148" spans="1:13">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>69</v>
       </c>
@@ -7861,7 +7867,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="149" spans="1:13">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>69</v>
       </c>
@@ -7890,7 +7896,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="150" spans="1:13">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>69</v>
       </c>
@@ -7919,7 +7925,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="151" spans="1:13">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>69</v>
       </c>
@@ -7948,7 +7954,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="152" spans="1:13">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>69</v>
       </c>
@@ -7986,7 +7992,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="153" spans="1:13">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>69</v>
       </c>
@@ -8021,7 +8027,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="154" spans="1:13">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A154">
         <v>69</v>
       </c>
@@ -8056,7 +8062,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="155" spans="1:13">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A155">
         <v>68</v>
       </c>
@@ -8085,7 +8091,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="156" spans="1:13">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A156">
         <v>68</v>
       </c>
@@ -8114,7 +8120,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="157" spans="1:13">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A157">
         <v>68</v>
       </c>
@@ -8143,7 +8149,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="158" spans="1:13">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A158">
         <v>67</v>
       </c>
@@ -8184,7 +8190,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="159" spans="1:13">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A159">
         <v>66</v>
       </c>
@@ -8213,7 +8219,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="160" spans="1:13">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A160">
         <v>66</v>
       </c>
@@ -8242,7 +8248,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="161" spans="1:13">
+    <row r="161" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>63</v>
       </c>
@@ -8271,7 +8277,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="162" spans="1:13">
+    <row r="162" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>62</v>
       </c>
@@ -8300,7 +8306,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="163" spans="1:13">
+    <row r="163" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>60</v>
       </c>
@@ -8329,7 +8335,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="164" spans="1:13">
+    <row r="164" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>59</v>
       </c>
@@ -8358,7 +8364,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="165" spans="1:13">
+    <row r="165" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>59</v>
       </c>
@@ -8387,7 +8393,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="166" spans="1:13">
+    <row r="166" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>59</v>
       </c>
@@ -8416,7 +8422,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="167" spans="1:13">
+    <row r="167" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A167">
         <v>58</v>
       </c>
@@ -8445,7 +8451,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="168" spans="1:13">
+    <row r="168" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A168">
         <v>58</v>
       </c>
@@ -8486,7 +8492,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="169" spans="1:13">
+    <row r="169" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A169">
         <v>57</v>
       </c>
@@ -8515,7 +8521,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="170" spans="1:13">
+    <row r="170" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A170">
         <v>57</v>
       </c>
@@ -8544,7 +8550,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="171" spans="1:13">
+    <row r="171" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A171">
         <v>57</v>
       </c>
@@ -8573,7 +8579,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="172" spans="1:13">
+    <row r="172" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A172">
         <v>56</v>
       </c>
@@ -8602,7 +8608,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="173" spans="1:13">
+    <row r="173" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A173">
         <v>56</v>
       </c>
@@ -8643,7 +8649,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="174" spans="1:13">
+    <row r="174" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A174">
         <v>56</v>
       </c>
@@ -8681,7 +8687,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="175" spans="1:13">
+    <row r="175" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A175">
         <v>56</v>
       </c>
@@ -8710,7 +8716,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="176" spans="1:13">
+    <row r="176" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A176">
         <v>55</v>
       </c>
@@ -8739,7 +8745,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="177" spans="1:13">
+    <row r="177" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A177">
         <v>54</v>
       </c>
@@ -8768,7 +8774,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="178" spans="1:13">
+    <row r="178" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A178">
         <v>53</v>
       </c>
@@ -8797,7 +8803,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="179" spans="1:13">
+    <row r="179" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A179">
         <v>52</v>
       </c>
@@ -8838,7 +8844,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="180" spans="1:13">
+    <row r="180" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A180">
         <v>50</v>
       </c>
@@ -8867,7 +8873,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="181" spans="1:13">
+    <row r="181" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A181">
         <v>50</v>
       </c>
@@ -8908,7 +8914,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="182" spans="1:13">
+    <row r="182" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A182">
         <v>50</v>
       </c>
@@ -8946,7 +8952,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="183" spans="1:13">
+    <row r="183" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A183">
         <v>50</v>
       </c>
@@ -8987,7 +8993,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="184" spans="1:13">
+    <row r="184" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A184">
         <v>50</v>
       </c>
@@ -9036,11 +9042,20 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CA1B76A-69BF-8C49-BD0C-404BACCDD367}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L107"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>472</v>
       </c>
@@ -9070,7 +9085,7 @@
       <c r="K1" s="5"/>
       <c r="L1" s="5"/>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>81</v>
       </c>
@@ -9096,7 +9111,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>81</v>
       </c>
@@ -9122,7 +9137,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>83</v>
       </c>
@@ -9148,7 +9163,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>87</v>
       </c>
@@ -9174,7 +9189,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>91</v>
       </c>
@@ -9200,7 +9215,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>92</v>
       </c>
@@ -9226,7 +9241,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>93</v>
       </c>
@@ -9252,7 +9267,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>93</v>
       </c>
@@ -9278,7 +9293,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>93</v>
       </c>
@@ -9304,7 +9319,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>93</v>
       </c>
@@ -9330,7 +9345,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>95</v>
       </c>
@@ -9356,7 +9371,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>94</v>
       </c>
@@ -9382,7 +9397,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>94</v>
       </c>
@@ -9408,7 +9423,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>94</v>
       </c>
@@ -9434,7 +9449,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>94</v>
       </c>
@@ -9460,7 +9475,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>97</v>
       </c>
@@ -9486,7 +9501,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>97</v>
       </c>
@@ -9512,7 +9527,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>96</v>
       </c>
@@ -9538,7 +9553,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>98</v>
       </c>
@@ -9564,7 +9579,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>100</v>
       </c>
@@ -9590,7 +9605,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>100</v>
       </c>
@@ -9616,7 +9631,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>100</v>
       </c>
@@ -9642,7 +9657,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>100</v>
       </c>
@@ -9668,7 +9683,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>100</v>
       </c>
@@ -9694,7 +9709,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>101</v>
       </c>
@@ -9720,7 +9735,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>101</v>
       </c>
@@ -9746,7 +9761,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>101</v>
       </c>
@@ -9772,7 +9787,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>101</v>
       </c>
@@ -9798,7 +9813,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>101</v>
       </c>
@@ -9824,7 +9839,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>102</v>
       </c>
@@ -9850,7 +9865,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>103</v>
       </c>
@@ -9876,7 +9891,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>105</v>
       </c>
@@ -9902,7 +9917,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>105</v>
       </c>
@@ -9928,7 +9943,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>110</v>
       </c>
@@ -9954,7 +9969,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>110</v>
       </c>
@@ -9980,7 +9995,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>110</v>
       </c>
@@ -10006,7 +10021,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>111</v>
       </c>
@@ -10032,7 +10047,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>111</v>
       </c>
@@ -10058,7 +10073,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>111</v>
       </c>
@@ -10084,7 +10099,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>112</v>
       </c>
@@ -10110,7 +10125,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>112</v>
       </c>
@@ -10136,7 +10151,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>114</v>
       </c>
@@ -10162,7 +10177,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>114</v>
       </c>
@@ -10188,7 +10203,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>115</v>
       </c>
@@ -10214,7 +10229,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>115</v>
       </c>
@@ -10240,7 +10255,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>115</v>
       </c>
@@ -10266,7 +10281,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>117</v>
       </c>
@@ -10292,7 +10307,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>118</v>
       </c>
@@ -10318,7 +10333,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>118</v>
       </c>
@@ -10344,7 +10359,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>123</v>
       </c>
@@ -10370,7 +10385,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:8">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>123</v>
       </c>
@@ -10396,7 +10411,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:8">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>123</v>
       </c>
@@ -10422,7 +10437,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54" spans="1:8">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>119</v>
       </c>
@@ -10448,7 +10463,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:8">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>126</v>
       </c>
@@ -10474,7 +10489,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>126</v>
       </c>
@@ -10500,7 +10515,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>126</v>
       </c>
@@ -10526,7 +10541,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:8">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>129</v>
       </c>
@@ -10552,7 +10567,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>129</v>
       </c>
@@ -10578,7 +10593,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:8">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>129</v>
       </c>
@@ -10604,7 +10619,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>129</v>
       </c>
@@ -10630,7 +10645,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="62" spans="1:8">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>129</v>
       </c>
@@ -10656,7 +10671,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>129</v>
       </c>
@@ -10682,7 +10697,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>130</v>
       </c>
@@ -10708,7 +10723,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="65" spans="1:8">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>130</v>
       </c>
@@ -10734,7 +10749,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:8">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>143</v>
       </c>
@@ -10760,7 +10775,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="67" spans="1:8">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>132</v>
       </c>
@@ -10786,7 +10801,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="1:8">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>138</v>
       </c>
@@ -10812,7 +10827,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="1:8">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>148</v>
       </c>
@@ -10838,7 +10853,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:8">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>148</v>
       </c>
@@ -10864,7 +10879,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="1:8">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>148</v>
       </c>
@@ -10890,7 +10905,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:8">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>148</v>
       </c>
@@ -10916,7 +10931,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="73" spans="1:8">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>148</v>
       </c>
@@ -10942,7 +10957,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="74" spans="1:8">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>148</v>
       </c>
@@ -10968,7 +10983,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>153</v>
       </c>
@@ -10994,7 +11009,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:8">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>153</v>
       </c>
@@ -11020,7 +11035,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="77" spans="1:8">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>153</v>
       </c>
@@ -11046,7 +11061,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="1:8">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>168</v>
       </c>
@@ -11072,7 +11087,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="79" spans="1:8">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>168</v>
       </c>
@@ -11098,7 +11113,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="80" spans="1:8">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>155</v>
       </c>
@@ -11124,7 +11139,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="81" spans="1:8">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>155</v>
       </c>
@@ -11150,7 +11165,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="82" spans="1:8">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>156</v>
       </c>
@@ -11176,7 +11191,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="83" spans="1:8">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>158</v>
       </c>
@@ -11202,7 +11217,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="84" spans="1:8">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>159</v>
       </c>
@@ -11228,7 +11243,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="85" spans="1:8">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>160</v>
       </c>
@@ -11254,7 +11269,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="86" spans="1:8">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>161</v>
       </c>
@@ -11280,7 +11295,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="87" spans="1:8">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>162</v>
       </c>
@@ -11306,7 +11321,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="88" spans="1:8">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>163</v>
       </c>
@@ -11332,7 +11347,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="89" spans="1:8">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>163</v>
       </c>
@@ -11358,7 +11373,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="90" spans="1:8">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>163</v>
       </c>
@@ -11384,7 +11399,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="91" spans="1:8">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>164</v>
       </c>
@@ -11410,7 +11425,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92" spans="1:8">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>167</v>
       </c>
@@ -11436,7 +11451,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="93" spans="1:8">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>166</v>
       </c>
@@ -11462,7 +11477,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="94" spans="1:8">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>169</v>
       </c>
@@ -11488,7 +11503,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="95" spans="1:8">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>171</v>
       </c>
@@ -11514,7 +11529,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="96" spans="1:8">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>172</v>
       </c>
@@ -11540,7 +11555,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="97" spans="1:8">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>172</v>
       </c>
@@ -11566,7 +11581,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="98" spans="1:8">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>172</v>
       </c>
@@ -11592,7 +11607,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="99" spans="1:8">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>175</v>
       </c>
@@ -11618,7 +11633,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="100" spans="1:8">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>175</v>
       </c>
@@ -11644,7 +11659,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="101" spans="1:8">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>175</v>
       </c>
@@ -11670,7 +11685,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="102" spans="1:8">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>175</v>
       </c>
@@ -11696,7 +11711,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="103" spans="1:8">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>176</v>
       </c>
@@ -11722,7 +11737,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="104" spans="1:8">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>176</v>
       </c>
@@ -11748,7 +11763,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105" spans="1:8">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>176</v>
       </c>
@@ -11774,7 +11789,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="106" spans="1:8">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>179</v>
       </c>
@@ -11800,7 +11815,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="107" spans="1:8">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>178</v>
       </c>
@@ -11832,12 +11847,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L84"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>472</v>
       </c>
@@ -11875,7 +11890,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>81</v>
       </c>
@@ -11913,7 +11928,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>81</v>
       </c>
@@ -11951,7 +11966,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>81</v>
       </c>
@@ -11986,7 +12001,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>81</v>
       </c>
@@ -12024,7 +12039,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>81</v>
       </c>
@@ -12059,7 +12074,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>81</v>
       </c>
@@ -12094,7 +12109,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>82</v>
       </c>
@@ -12132,7 +12147,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>83</v>
       </c>
@@ -12170,7 +12185,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>83</v>
       </c>
@@ -12208,7 +12223,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>83</v>
       </c>
@@ -12246,7 +12261,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>83</v>
       </c>
@@ -12281,7 +12296,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>84</v>
       </c>
@@ -12319,7 +12334,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>84</v>
       </c>
@@ -12357,7 +12372,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>86</v>
       </c>
@@ -12395,7 +12410,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>86</v>
       </c>
@@ -12433,7 +12448,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:12">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>86</v>
       </c>
@@ -12471,7 +12486,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:12">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>86</v>
       </c>
@@ -12509,7 +12524,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:12">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>86</v>
       </c>
@@ -12547,7 +12562,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:12">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>86</v>
       </c>
@@ -12585,7 +12600,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:12">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>88</v>
       </c>
@@ -12617,7 +12632,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>88</v>
       </c>
@@ -12652,7 +12667,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>89</v>
       </c>
@@ -12690,7 +12705,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:12">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>89</v>
       </c>
@@ -12728,7 +12743,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:12">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>91</v>
       </c>
@@ -12766,7 +12781,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:12">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>91</v>
       </c>
@@ -12804,7 +12819,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:12">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>91</v>
       </c>
@@ -12842,7 +12857,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:12">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>91</v>
       </c>
@@ -12880,7 +12895,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:12">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>90</v>
       </c>
@@ -12918,7 +12933,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:12">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>93</v>
       </c>
@@ -12956,7 +12971,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>93</v>
       </c>
@@ -12994,7 +13009,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:12">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>95</v>
       </c>
@@ -13029,7 +13044,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:12">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>95</v>
       </c>
@@ -13064,7 +13079,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:12">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>97</v>
       </c>
@@ -13102,7 +13117,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:12">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>96</v>
       </c>
@@ -13137,7 +13152,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:12">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>96</v>
       </c>
@@ -13172,7 +13187,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:12">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>99</v>
       </c>
@@ -13210,7 +13225,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:12">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>101</v>
       </c>
@@ -13248,7 +13263,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:12">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>104</v>
       </c>
@@ -13283,7 +13298,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:12">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>106</v>
       </c>
@@ -13321,7 +13336,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:12">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>105</v>
       </c>
@@ -13356,7 +13371,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:12">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>108</v>
       </c>
@@ -13391,7 +13406,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:12">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>108</v>
       </c>
@@ -13426,7 +13441,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:12">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>116</v>
       </c>
@@ -13461,7 +13476,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:12">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>116</v>
       </c>
@@ -13496,7 +13511,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46" spans="1:12">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>117</v>
       </c>
@@ -13534,7 +13549,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:12">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>117</v>
       </c>
@@ -13572,7 +13587,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48" spans="1:12">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>118</v>
       </c>
@@ -13610,7 +13625,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:12">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>119</v>
       </c>
@@ -13645,7 +13660,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:12">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>119</v>
       </c>
@@ -13680,7 +13695,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51" spans="1:12">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>119</v>
       </c>
@@ -13715,7 +13730,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:12">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>119</v>
       </c>
@@ -13750,7 +13765,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:12">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>119</v>
       </c>
@@ -13788,7 +13803,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54" spans="1:12">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>121</v>
       </c>
@@ -13826,7 +13841,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:12">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>121</v>
       </c>
@@ -13864,7 +13879,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:12">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>120</v>
       </c>
@@ -13899,7 +13914,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:12">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>124</v>
       </c>
@@ -13937,7 +13952,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:12">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>124</v>
       </c>
@@ -13975,7 +13990,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="1:12">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>122</v>
       </c>
@@ -14010,7 +14025,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:12">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>122</v>
       </c>
@@ -14048,7 +14063,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:12">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>122</v>
       </c>
@@ -14083,7 +14098,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="62" spans="1:12">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>122</v>
       </c>
@@ -14118,7 +14133,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:12">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>122</v>
       </c>
@@ -14153,7 +14168,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="64" spans="1:12">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>125</v>
       </c>
@@ -14191,7 +14206,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="65" spans="1:12">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>125</v>
       </c>
@@ -14229,7 +14244,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:12">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>133</v>
       </c>
@@ -14264,7 +14279,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="67" spans="1:12">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>136</v>
       </c>
@@ -14302,7 +14317,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="1:12">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>139</v>
       </c>
@@ -14340,7 +14355,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="1:12">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>144</v>
       </c>
@@ -14378,7 +14393,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:12">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>150</v>
       </c>
@@ -14416,7 +14431,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="1:12">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>154</v>
       </c>
@@ -14451,7 +14466,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:12">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>164</v>
       </c>
@@ -14489,7 +14504,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="1:12">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>173</v>
       </c>
@@ -14524,7 +14539,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74" spans="1:12">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>179</v>
       </c>
@@ -14562,7 +14577,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="1:12">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>122</v>
       </c>
@@ -14597,7 +14612,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:12">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>125</v>
       </c>
@@ -14635,7 +14650,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="77" spans="1:12">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>125</v>
       </c>
@@ -14673,7 +14688,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="1:12">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>133</v>
       </c>
@@ -14708,7 +14723,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="1:12">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>136</v>
       </c>
@@ -14746,7 +14761,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:12">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>139</v>
       </c>
@@ -14784,7 +14799,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="81" spans="1:12">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>144</v>
       </c>
@@ -14822,7 +14837,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="1:12">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>150</v>
       </c>
@@ -14860,7 +14875,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:12">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>154</v>
       </c>
@@ -14895,7 +14910,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:12">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>164</v>
       </c>

</xml_diff>